<commit_message>
Refresh sample cases for new plot controls
</commit_message>
<xml_diff>
--- a/samples/sample_01_temp_c_to_k.xlsx
+++ b/samples/sample_01_temp_c_to_k.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="sample" sheetId="1" r:id="Raca54b0430094e0c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="sample" sheetId="1" r:id="Rd60ac25e6e254144"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -293,7 +293,7 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="5" t="str">
-        <x:v>练习：绘制多条 emission curve，比较低浓度、高浓度和参考样品的峰形差异。</x:v>
+        <x:v>练习：预设会启用末端标签、平滑连接、手动轴范围和峰位参考线。</x:v>
       </x:c>
       <x:c r="B3" s="5" t="str"/>
       <x:c r="C3" s="5" t="str"/>
@@ -302,7 +302,7 @@
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="5" t="str">
-        <x:v>建议：X 轴为 wavelength_nm，Y 轴加入 sample_low_a_u、sample_high_a_u、reference_a_u。</x:v>
+        <x:v>建议：X 轴为 wavelength_nm，三条 Y 曲线用于比较峰形和强度。</x:v>
       </x:c>
       <x:c r="B4" s="5" t="str"/>
       <x:c r="C4" s="5" t="str"/>

</xml_diff>